<commit_message>
feat(feedback): add scoring setup and analytics features
- Introduced ScoringSetup.module.css for styling the scoring setup panel.
- Added scorePreview.json fixture for testing various scoring scenarios.
- Created feedbackCharts.module.css for chart styling in feedback analytics.
- Implemented feedbackDashboardData.ts for handling feedback dashboard data and date formatting.
- Added lectureAnalyticsLabels.ts for generating labels for lecture analytics.
- Developed questionAnalyticsConfig.ts and questionAnalyticsConfig.test.ts for managing question analytics settings and ensuring configuration integrity.
- Implemented scoreClassification.ts for classifying feedback scores.
- Created scorePreview.ts and scorePreview.test.ts for previewing scores and validating scoring logic.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/post-lecture-question-bank.xlsx
+++ b/frontend/public/templates/post-lecture-question-bank.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="R0745a93f00494411"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="R923400e3fc474cdd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -339,6 +339,7 @@
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -368,6 +369,9 @@
       </x:c>
       <x:c r="I1" s="10" t="str">
         <x:v>Option 6</x:v>
+      </x:c>
+      <x:c r="J1" s="10" t="str">
+        <x:v>Importance</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
@@ -386,6 +390,9 @@
       <x:c r="G2" s="2" t="str"/>
       <x:c r="H2" s="2" t="str"/>
       <x:c r="I2" s="2" t="str"/>
+      <x:c r="J2" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -403,6 +410,9 @@
       <x:c r="G3" s="2" t="str"/>
       <x:c r="H3" s="2" t="str"/>
       <x:c r="I3" s="2" t="str"/>
+      <x:c r="J3" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -420,6 +430,9 @@
       <x:c r="G4" s="2" t="str"/>
       <x:c r="H4" s="2" t="str"/>
       <x:c r="I4" s="2" t="str"/>
+      <x:c r="J4" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -437,6 +450,9 @@
       <x:c r="G5" s="2" t="str"/>
       <x:c r="H5" s="2" t="str"/>
       <x:c r="I5" s="2" t="str"/>
+      <x:c r="J5" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -454,6 +470,9 @@
       <x:c r="G6" s="2" t="str"/>
       <x:c r="H6" s="2" t="str"/>
       <x:c r="I6" s="2" t="str"/>
+      <x:c r="J6" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -477,6 +496,9 @@
       <x:c r="G7" s="2" t="str"/>
       <x:c r="H7" s="2" t="str"/>
       <x:c r="I7" s="2" t="str"/>
+      <x:c r="J7" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
       <x:c r="A8" s="12" t="str">
@@ -494,11 +516,17 @@
       <x:c r="G8" s="2" t="str"/>
       <x:c r="H8" s="2" t="str"/>
       <x:c r="I8" s="2" t="str"/>
+      <x:c r="J8" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C2:C1001">
       <x:formula1>"5 Stars,Written answer,Short answer,Yes / No,Choose one,Choose several,Dropdown list,Number rating,Agreement scale,Number,Date,Full name,Email address,Photo upload"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J2:J1001">
+      <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: enforce scoring requirements for eligible questions and improve analytics setup
- Added tests to ensure scoring is required for single choice, multiple choice, dropdown, and likert questions even when excluded from overall scoring.
- Updated QuestionAnalyticsSettings component to handle scoring setup more robustly, including clearer messaging for incomplete setups.
- Enhanced QuestionBankImport to report questions needing scoring setup before publishing.
- Improved error handling and validation for scoring configurations in post-lecture question bank imports.
- Refactored scoring readiness checks to provide clearer feedback on unscored and incomplete questions.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/post-lecture-question-bank.xlsx
+++ b/frontend/public/templates/post-lecture-question-bank.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="R923400e3fc474cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="R5c75581197f843b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="0.##"/>
+    <x:numFmt numFmtId="201" formatCode="0.00"/>
+  </x:numFmts>
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -29,8 +33,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF172554"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -40,6 +49,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF541EA0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFBEB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFBEB"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -89,7 +108,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -127,6 +146,37 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -340,9 +390,28 @@
     <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="17" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="17" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="17" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="17" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="17" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="17" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="17" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="17" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="17" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="17" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="8" t="str">
         <x:v>Category</x:v>
       </x:c>
@@ -373,8 +442,65 @@
       <x:c r="J1" s="10" t="str">
         <x:v>Importance</x:v>
       </x:c>
+      <x:c r="K1" s="14" t="str">
+        <x:v>Scoring</x:v>
+      </x:c>
+      <x:c r="L1" s="14" t="str">
+        <x:v>Yes score</x:v>
+      </x:c>
+      <x:c r="M1" s="14" t="str">
+        <x:v>No score</x:v>
+      </x:c>
+      <x:c r="N1" s="14" t="str">
+        <x:v>Option 1 score</x:v>
+      </x:c>
+      <x:c r="O1" s="14" t="str">
+        <x:v>Option 2 score</x:v>
+      </x:c>
+      <x:c r="P1" s="14" t="str">
+        <x:v>Option 3 score</x:v>
+      </x:c>
+      <x:c r="Q1" s="14" t="str">
+        <x:v>Option 4 score</x:v>
+      </x:c>
+      <x:c r="R1" s="14" t="str">
+        <x:v>Option 5 score</x:v>
+      </x:c>
+      <x:c r="S1" s="14" t="str">
+        <x:v>Option 6 score</x:v>
+      </x:c>
+      <x:c r="T1" s="14" t="str">
+        <x:v>Score min</x:v>
+      </x:c>
+      <x:c r="U1" s="14" t="str">
+        <x:v>Score max</x:v>
+      </x:c>
+      <x:c r="V1" s="14" t="str">
+        <x:v>Include in overall score</x:v>
+      </x:c>
+      <x:c r="W1" s="14" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="X1" s="14" t="str">
+        <x:v>Help text</x:v>
+      </x:c>
+      <x:c r="Y1" s="14" t="str">
+        <x:v>Scale max</x:v>
+      </x:c>
+      <x:c r="Z1" s="14" t="str">
+        <x:v>Scale display</x:v>
+      </x:c>
+      <x:c r="AA1" s="14" t="str">
+        <x:v>Scale labels</x:v>
+      </x:c>
+      <x:c r="AB1" s="14" t="str">
+        <x:v>Min label</x:v>
+      </x:c>
+      <x:c r="AC1" s="14" t="str">
+        <x:v>Max label</x:v>
+      </x:c>
     </x:row>
-    <x:row r="2" ht="32" customHeight="1">
+    <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="12" t="str">
         <x:v>Teaching</x:v>
       </x:c>
@@ -384,17 +510,42 @@
       <x:c r="C2" s="12" t="str">
         <x:v>5 Stars</x:v>
       </x:c>
-      <x:c r="D2" s="2" t="str"/>
-      <x:c r="E2" s="2" t="str"/>
-      <x:c r="F2" s="2" t="str"/>
-      <x:c r="G2" s="2" t="str"/>
-      <x:c r="H2" s="2" t="str"/>
-      <x:c r="I2" s="2" t="str"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
       <x:c r="J2" s="12" t="str">
         <x:v>Medium</x:v>
       </x:c>
+      <x:c r="K2" s="22" t="str">
+        <x:v>Higher is better</x:v>
+      </x:c>
+      <x:c r="L2" s="24"/>
+      <x:c r="M2" s="24"/>
+      <x:c r="N2" s="24"/>
+      <x:c r="O2" s="24"/>
+      <x:c r="P2" s="24"/>
+      <x:c r="Q2" s="24"/>
+      <x:c r="R2" s="24"/>
+      <x:c r="S2" s="24"/>
+      <x:c r="T2" s="24"/>
+      <x:c r="U2" s="24"/>
+      <x:c r="V2" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W2" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X2" s="22"/>
+      <x:c r="Y2" s="22"/>
+      <x:c r="Z2" s="22"/>
+      <x:c r="AA2" s="22"/>
+      <x:c r="AB2" s="22"/>
+      <x:c r="AC2" s="22"/>
     </x:row>
-    <x:row r="3" ht="32" customHeight="1">
+    <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="12" t="str">
         <x:v>Teaching</x:v>
       </x:c>
@@ -404,17 +555,42 @@
       <x:c r="C3" s="12" t="str">
         <x:v>5 Stars</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="str"/>
-      <x:c r="E3" s="2" t="str"/>
-      <x:c r="F3" s="2" t="str"/>
-      <x:c r="G3" s="2" t="str"/>
-      <x:c r="H3" s="2" t="str"/>
-      <x:c r="I3" s="2" t="str"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
       <x:c r="J3" s="12" t="str">
         <x:v>Medium</x:v>
       </x:c>
+      <x:c r="K3" s="22" t="str">
+        <x:v>Higher is better</x:v>
+      </x:c>
+      <x:c r="L3" s="24"/>
+      <x:c r="M3" s="24"/>
+      <x:c r="N3" s="24"/>
+      <x:c r="O3" s="24"/>
+      <x:c r="P3" s="24"/>
+      <x:c r="Q3" s="24"/>
+      <x:c r="R3" s="24"/>
+      <x:c r="S3" s="24"/>
+      <x:c r="T3" s="24"/>
+      <x:c r="U3" s="24"/>
+      <x:c r="V3" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W3" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X3" s="22"/>
+      <x:c r="Y3" s="22"/>
+      <x:c r="Z3" s="22"/>
+      <x:c r="AA3" s="22"/>
+      <x:c r="AB3" s="22"/>
+      <x:c r="AC3" s="22"/>
     </x:row>
-    <x:row r="4" ht="32" customHeight="1">
+    <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="12" t="str">
         <x:v>Teaching</x:v>
       </x:c>
@@ -424,17 +600,46 @@
       <x:c r="C4" s="12" t="str">
         <x:v>Yes / No</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="str"/>
-      <x:c r="E4" s="2" t="str"/>
-      <x:c r="F4" s="2" t="str"/>
-      <x:c r="G4" s="2" t="str"/>
-      <x:c r="H4" s="2" t="str"/>
-      <x:c r="I4" s="2" t="str"/>
+      <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
+      <x:c r="I4" s="2"/>
       <x:c r="J4" s="12" t="str">
         <x:v>Medium</x:v>
       </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>Per answer</x:v>
+      </x:c>
+      <x:c r="L4" s="24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M4" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N4" s="24"/>
+      <x:c r="O4" s="24"/>
+      <x:c r="P4" s="24"/>
+      <x:c r="Q4" s="24"/>
+      <x:c r="R4" s="24"/>
+      <x:c r="S4" s="24"/>
+      <x:c r="T4" s="24"/>
+      <x:c r="U4" s="24"/>
+      <x:c r="V4" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W4" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X4" s="22"/>
+      <x:c r="Y4" s="22"/>
+      <x:c r="Z4" s="22"/>
+      <x:c r="AA4" s="22"/>
+      <x:c r="AB4" s="22"/>
+      <x:c r="AC4" s="22"/>
     </x:row>
-    <x:row r="5" ht="32" customHeight="1">
+    <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>Resources</x:v>
       </x:c>
@@ -444,17 +649,42 @@
       <x:c r="C5" s="12" t="str">
         <x:v>5 Stars</x:v>
       </x:c>
-      <x:c r="D5" s="2" t="str"/>
-      <x:c r="E5" s="2" t="str"/>
-      <x:c r="F5" s="2" t="str"/>
-      <x:c r="G5" s="2" t="str"/>
-      <x:c r="H5" s="2" t="str"/>
-      <x:c r="I5" s="2" t="str"/>
+      <x:c r="D5" s="2"/>
+      <x:c r="E5" s="2"/>
+      <x:c r="F5" s="2"/>
+      <x:c r="G5" s="2"/>
+      <x:c r="H5" s="2"/>
+      <x:c r="I5" s="2"/>
       <x:c r="J5" s="12" t="str">
         <x:v>Medium</x:v>
       </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>Higher is better</x:v>
+      </x:c>
+      <x:c r="L5" s="24"/>
+      <x:c r="M5" s="24"/>
+      <x:c r="N5" s="24"/>
+      <x:c r="O5" s="24"/>
+      <x:c r="P5" s="24"/>
+      <x:c r="Q5" s="24"/>
+      <x:c r="R5" s="24"/>
+      <x:c r="S5" s="24"/>
+      <x:c r="T5" s="24"/>
+      <x:c r="U5" s="24"/>
+      <x:c r="V5" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W5" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X5" s="22"/>
+      <x:c r="Y5" s="22"/>
+      <x:c r="Z5" s="22"/>
+      <x:c r="AA5" s="22"/>
+      <x:c r="AB5" s="22"/>
+      <x:c r="AC5" s="22"/>
     </x:row>
-    <x:row r="6" ht="32" customHeight="1">
+    <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>Resources</x:v>
       </x:c>
@@ -464,17 +694,42 @@
       <x:c r="C6" s="12" t="str">
         <x:v>5 Stars</x:v>
       </x:c>
-      <x:c r="D6" s="2" t="str"/>
-      <x:c r="E6" s="2" t="str"/>
-      <x:c r="F6" s="2" t="str"/>
-      <x:c r="G6" s="2" t="str"/>
-      <x:c r="H6" s="2" t="str"/>
-      <x:c r="I6" s="2" t="str"/>
+      <x:c r="D6" s="2"/>
+      <x:c r="E6" s="2"/>
+      <x:c r="F6" s="2"/>
+      <x:c r="G6" s="2"/>
+      <x:c r="H6" s="2"/>
+      <x:c r="I6" s="2"/>
       <x:c r="J6" s="12" t="str">
         <x:v>Medium</x:v>
       </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>Higher is better</x:v>
+      </x:c>
+      <x:c r="L6" s="24"/>
+      <x:c r="M6" s="24"/>
+      <x:c r="N6" s="24"/>
+      <x:c r="O6" s="24"/>
+      <x:c r="P6" s="24"/>
+      <x:c r="Q6" s="24"/>
+      <x:c r="R6" s="24"/>
+      <x:c r="S6" s="24"/>
+      <x:c r="T6" s="24"/>
+      <x:c r="U6" s="24"/>
+      <x:c r="V6" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W6" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X6" s="22"/>
+      <x:c r="Y6" s="22"/>
+      <x:c r="Z6" s="22"/>
+      <x:c r="AA6" s="22"/>
+      <x:c r="AB6" s="22"/>
+      <x:c r="AC6" s="22"/>
     </x:row>
-    <x:row r="7" ht="32" customHeight="1">
+    <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="12" t="str">
         <x:v>Resources</x:v>
       </x:c>
@@ -493,14 +748,45 @@
       <x:c r="F7" s="12" t="str">
         <x:v>Practice</x:v>
       </x:c>
-      <x:c r="G7" s="2" t="str"/>
-      <x:c r="H7" s="2" t="str"/>
-      <x:c r="I7" s="2" t="str"/>
+      <x:c r="G7" s="2"/>
+      <x:c r="H7" s="2"/>
+      <x:c r="I7" s="2"/>
       <x:c r="J7" s="12" t="str">
         <x:v>Medium</x:v>
       </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>Per answer</x:v>
+      </x:c>
+      <x:c r="L7" s="24"/>
+      <x:c r="M7" s="24"/>
+      <x:c r="N7" s="24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O7" s="24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P7" s="24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="Q7" s="24"/>
+      <x:c r="R7" s="24"/>
+      <x:c r="S7" s="24"/>
+      <x:c r="T7" s="24"/>
+      <x:c r="U7" s="24"/>
+      <x:c r="V7" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W7" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X7" s="22"/>
+      <x:c r="Y7" s="22"/>
+      <x:c r="Z7" s="22"/>
+      <x:c r="AA7" s="22"/>
+      <x:c r="AB7" s="22"/>
+      <x:c r="AC7" s="22"/>
     </x:row>
-    <x:row r="8" ht="32" customHeight="1">
+    <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="12" t="str">
         <x:v>General</x:v>
       </x:c>
@@ -510,23 +796,142 @@
       <x:c r="C8" s="12" t="str">
         <x:v>Written answer</x:v>
       </x:c>
-      <x:c r="D8" s="2" t="str"/>
-      <x:c r="E8" s="2" t="str"/>
-      <x:c r="F8" s="2" t="str"/>
-      <x:c r="G8" s="2" t="str"/>
-      <x:c r="H8" s="2" t="str"/>
-      <x:c r="I8" s="2" t="str"/>
+      <x:c r="D8" s="2"/>
+      <x:c r="E8" s="2"/>
+      <x:c r="F8" s="2"/>
+      <x:c r="G8" s="2"/>
+      <x:c r="H8" s="2"/>
+      <x:c r="I8" s="2"/>
       <x:c r="J8" s="12" t="str">
         <x:v>Medium</x:v>
       </x:c>
+      <x:c r="K8" s="22"/>
+      <x:c r="L8" s="24"/>
+      <x:c r="M8" s="24"/>
+      <x:c r="N8" s="24"/>
+      <x:c r="O8" s="24"/>
+      <x:c r="P8" s="24"/>
+      <x:c r="Q8" s="24"/>
+      <x:c r="R8" s="24"/>
+      <x:c r="S8" s="24"/>
+      <x:c r="T8" s="24"/>
+      <x:c r="U8" s="24"/>
+      <x:c r="V8" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W8" s="22" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X8" s="22"/>
+      <x:c r="Y8" s="22"/>
+      <x:c r="Z8" s="22"/>
+      <x:c r="AA8" s="22"/>
+      <x:c r="AB8" s="22"/>
+      <x:c r="AC8" s="22"/>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="12" t="str">
+        <x:v>Practice</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="str">
+        <x:v>How many practice tasks did you complete?</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="D9" s="12"/>
+      <x:c r="E9" s="12"/>
+      <x:c r="F9" s="12"/>
+      <x:c r="G9" s="2"/>
+      <x:c r="H9" s="2"/>
+      <x:c r="I9" s="2"/>
+      <x:c r="J9" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>Higher is better</x:v>
+      </x:c>
+      <x:c r="L9" s="24"/>
+      <x:c r="M9" s="24"/>
+      <x:c r="N9" s="24"/>
+      <x:c r="O9" s="24"/>
+      <x:c r="P9" s="24"/>
+      <x:c r="Q9" s="24"/>
+      <x:c r="R9" s="24"/>
+      <x:c r="S9" s="24"/>
+      <x:c r="T9" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U9" s="24" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V9" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W9" s="22" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X9" s="22"/>
+      <x:c r="Y9" s="22"/>
+      <x:c r="Z9" s="22"/>
+      <x:c r="AA9" s="22"/>
+      <x:c r="AB9" s="22"/>
+      <x:c r="AC9" s="22"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="15">
     <x:dataValidation type="list" sqref="C2:C1001">
       <x:formula1>"5 Stars,Written answer,Short answer,Yes / No,Choose one,Choose several,Dropdown list,Number rating,Agreement scale,Number,Date,Full name,Email address,Photo upload"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J2:J1001">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K2:K1001">
+      <x:formula1>"Higher is better,Lower is better,Per answer,Not scored"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="V2:V1001">
+      <x:formula1>"Yes,No"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="W2:W1001">
+      <x:formula1>"Yes,No"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="L2:L1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="M2:M1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="N2:N1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="O2:O1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="P2:P1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="Q2:Q1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="R2:R1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="S2:S1001">
+      <x:formula1>0</x:formula1>
+      <x:formula2>100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="Y2:Y1001">
+      <x:formula1>"5,10"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="Z2:Z1001">
+      <x:formula1>"stars,numbers"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>